<commit_message>
Update roadmap data from Excel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/roadmap.xlsx
+++ b/data/roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/akhilbhaskaruni/Desktop/ai-roadmap-web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED27D42A-59F3-7545-9546-82BB99C5BFB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ECE66A7-F706-CF48-8121-4304C3690240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="95">
   <si>
     <t>id</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t>Abhilasha</t>
+  </si>
+  <si>
+    <t>Dummy project 2</t>
   </si>
 </sst>
 </file>
@@ -692,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -861,6 +864,36 @@
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H6" s="4">
+        <v>45750</v>
+      </c>
+      <c r="I6" s="4">
+        <v>45834</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>